<commit_message>
Add razon de devolucion to facturacion and backend
</commit_message>
<xml_diff>
--- a/Analisis CFBC MAYO-JUNIO.xlsx
+++ b/Analisis CFBC MAYO-JUNIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yisus\Desktop\APLICACION CHOFERES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986B1B6D-232C-4110-8DDE-FFBBDA950B1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5FBE737-8DC0-4CBD-8086-2F15AAEADAA9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="58">
   <si>
     <t>Salida</t>
   </si>
@@ -759,7 +759,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:L851"/>
+  <dimension ref="A1:L905"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="11" bestFit="1" customWidth="1"/>
@@ -25406,7 +25406,7 @@
         <v>177</v>
       </c>
       <c r="L837" s="9">
-        <f t="shared" ref="L837:L851" si="14">K837*J837</f>
+        <f t="shared" ref="L837:L900" si="14">K837*J837</f>
         <v>3186</v>
       </c>
     </row>
@@ -25814,6 +25814,1572 @@
       <c r="L851" s="9">
         <f t="shared" si="14"/>
         <v>1512</v>
+      </c>
+    </row>
+    <row r="852" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A852" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F852" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G852, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G852" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H852" s="2">
+        <v>816</v>
+      </c>
+      <c r="I852" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J852" s="4">
+        <v>8</v>
+      </c>
+      <c r="K852" s="8">
+        <f>IFERROR(VLOOKUP(I852, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L852" s="9">
+        <f t="shared" si="14"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="853" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A853" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F853" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G853, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G853" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H853" s="2">
+        <v>816</v>
+      </c>
+      <c r="I853" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J853" s="4">
+        <v>10</v>
+      </c>
+      <c r="K853" s="8">
+        <f>IFERROR(VLOOKUP(I853, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L853" s="9">
+        <f t="shared" si="14"/>
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="854" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A854" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F854" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G854, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G854" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H854" s="2">
+        <v>816</v>
+      </c>
+      <c r="I854" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J854" s="4">
+        <v>8</v>
+      </c>
+      <c r="K854" s="8">
+        <f>IFERROR(VLOOKUP(I854, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L854" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="855" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A855" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F855" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G855, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G855" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H855" s="2">
+        <v>816</v>
+      </c>
+      <c r="I855" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J855" s="4">
+        <v>6</v>
+      </c>
+      <c r="K855" s="8">
+        <f>IFERROR(VLOOKUP(I855, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>177</v>
+      </c>
+      <c r="L855" s="9">
+        <f t="shared" si="14"/>
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="856" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A856" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F856" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G856, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G856" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H856" s="2">
+        <v>816</v>
+      </c>
+      <c r="I856" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J856" s="4">
+        <v>10</v>
+      </c>
+      <c r="K856" s="8">
+        <f>IFERROR(VLOOKUP(I856, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L856" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="857" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A857" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F857" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G857, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PLAYAS DE TIJUANA</v>
+      </c>
+      <c r="G857" s="1">
+        <v>1613</v>
+      </c>
+      <c r="H857" s="2">
+        <v>816</v>
+      </c>
+      <c r="I857" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J857" s="4">
+        <v>16</v>
+      </c>
+      <c r="K857" s="8">
+        <f>IFERROR(VLOOKUP(I857, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L857" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="858" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A858" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F858" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G858, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PACIFICO</v>
+      </c>
+      <c r="G858" s="1">
+        <v>1616</v>
+      </c>
+      <c r="H858" s="2">
+        <v>817</v>
+      </c>
+      <c r="I858" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J858" s="4">
+        <v>10</v>
+      </c>
+      <c r="K858" s="8">
+        <f>IFERROR(VLOOKUP(I858, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L858" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="859" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A859" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F859" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G859, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC PACIFICO</v>
+      </c>
+      <c r="G859" s="1">
+        <v>1616</v>
+      </c>
+      <c r="H859" s="2">
+        <v>817</v>
+      </c>
+      <c r="I859" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J859" s="4">
+        <v>16</v>
+      </c>
+      <c r="K859" s="8">
+        <f>IFERROR(VLOOKUP(I859, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L859" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="860" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A860" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F860" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G860, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC LOMAS DE SANTA FE</v>
+      </c>
+      <c r="G860" s="1">
+        <v>190</v>
+      </c>
+      <c r="H860" s="2">
+        <v>818</v>
+      </c>
+      <c r="I860" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J860" s="4">
+        <v>8</v>
+      </c>
+      <c r="K860" s="8">
+        <f>IFERROR(VLOOKUP(I860, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L860" s="9">
+        <f t="shared" si="14"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="861" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A861" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F861" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G861, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC LOMAS DE SANTA FE</v>
+      </c>
+      <c r="G861" s="1">
+        <v>190</v>
+      </c>
+      <c r="H861" s="2">
+        <v>818</v>
+      </c>
+      <c r="I861" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J861" s="4">
+        <v>8</v>
+      </c>
+      <c r="K861" s="8">
+        <f>IFERROR(VLOOKUP(I861, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L861" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="862" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A862" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F862" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G862, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC LOMAS DE SANTA FE</v>
+      </c>
+      <c r="G862" s="1">
+        <v>190</v>
+      </c>
+      <c r="H862" s="2">
+        <v>818</v>
+      </c>
+      <c r="I862" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J862" s="4">
+        <v>10</v>
+      </c>
+      <c r="K862" s="8">
+        <f>IFERROR(VLOOKUP(I862, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L862" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="863" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A863" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F863" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G863, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC LOMAS DE SANTA FE</v>
+      </c>
+      <c r="G863" s="1">
+        <v>190</v>
+      </c>
+      <c r="H863" s="2">
+        <v>818</v>
+      </c>
+      <c r="I863" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J863" s="4">
+        <v>16</v>
+      </c>
+      <c r="K863" s="8">
+        <f>IFERROR(VLOOKUP(I863, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L863" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="864" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A864" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F864" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G864, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G864" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H864" s="2">
+        <v>819</v>
+      </c>
+      <c r="I864" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J864" s="4">
+        <v>4</v>
+      </c>
+      <c r="K864" s="8">
+        <f>IFERROR(VLOOKUP(I864, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L864" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="865" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A865" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F865" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G865, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G865" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H865" s="2">
+        <v>819</v>
+      </c>
+      <c r="I865" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J865" s="4">
+        <v>6</v>
+      </c>
+      <c r="K865" s="8">
+        <f>IFERROR(VLOOKUP(I865, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L865" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="866" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A866" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F866" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G866, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G866" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H866" s="2">
+        <v>819</v>
+      </c>
+      <c r="I866" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J866" s="4">
+        <v>16</v>
+      </c>
+      <c r="K866" s="8">
+        <f>IFERROR(VLOOKUP(I866, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L866" s="9">
+        <f t="shared" si="14"/>
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="867" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A867" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F867" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G867, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G867" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H867" s="2">
+        <v>819</v>
+      </c>
+      <c r="I867" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J867" s="4">
+        <v>10</v>
+      </c>
+      <c r="K867" s="8">
+        <f>IFERROR(VLOOKUP(I867, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L867" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="868" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A868" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F868" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G868, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G868" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H868" s="2">
+        <v>819</v>
+      </c>
+      <c r="I868" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J868" s="4">
+        <v>16</v>
+      </c>
+      <c r="K868" s="8">
+        <f>IFERROR(VLOOKUP(I868, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L868" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="869" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A869" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F869" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G869, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G869" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H869" s="2">
+        <v>820</v>
+      </c>
+      <c r="I869" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J869" s="4">
+        <v>4</v>
+      </c>
+      <c r="K869" s="8">
+        <f>IFERROR(VLOOKUP(I869, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L869" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="870" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A870" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F870" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G870, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G870" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H870" s="2">
+        <v>820</v>
+      </c>
+      <c r="I870" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J870" s="4">
+        <v>6</v>
+      </c>
+      <c r="K870" s="8">
+        <f>IFERROR(VLOOKUP(I870, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L870" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="871" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A871" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F871" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G871, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G871" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H871" s="2">
+        <v>820</v>
+      </c>
+      <c r="I871" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J871" s="4">
+        <v>8</v>
+      </c>
+      <c r="K871" s="8">
+        <f>IFERROR(VLOOKUP(I871, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L871" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="872" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A872" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F872" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G872, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G872" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H872" s="2">
+        <v>820</v>
+      </c>
+      <c r="I872" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J872" s="4">
+        <v>16</v>
+      </c>
+      <c r="K872" s="8">
+        <f>IFERROR(VLOOKUP(I872, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L872" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="873" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A873" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F873" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G873, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G873" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H873" s="2">
+        <v>821</v>
+      </c>
+      <c r="I873" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J873" s="4">
+        <v>4</v>
+      </c>
+      <c r="K873" s="8">
+        <f>IFERROR(VLOOKUP(I873, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L873" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="874" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A874" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F874" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G874, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G874" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H874" s="2">
+        <v>821</v>
+      </c>
+      <c r="I874" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J874" s="4">
+        <v>6</v>
+      </c>
+      <c r="K874" s="8">
+        <f>IFERROR(VLOOKUP(I874, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L874" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="875" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A875" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F875" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G875, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G875" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H875" s="2">
+        <v>821</v>
+      </c>
+      <c r="I875" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J875" s="4">
+        <v>8</v>
+      </c>
+      <c r="K875" s="8">
+        <f>IFERROR(VLOOKUP(I875, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L875" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="876" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A876" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F876" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G876, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G876" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H876" s="2">
+        <v>821</v>
+      </c>
+      <c r="I876" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J876" s="4">
+        <v>10</v>
+      </c>
+      <c r="K876" s="8">
+        <f>IFERROR(VLOOKUP(I876, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L876" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="877" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A877" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F877" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G877, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G877" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H877" s="2">
+        <v>821</v>
+      </c>
+      <c r="I877" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J877" s="4">
+        <v>16</v>
+      </c>
+      <c r="K877" s="8">
+        <f>IFERROR(VLOOKUP(I877, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L877" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="878" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A878" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F878" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G878, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA 2000</v>
+      </c>
+      <c r="G878" s="1">
+        <v>4155</v>
+      </c>
+      <c r="H878" s="2">
+        <v>822</v>
+      </c>
+      <c r="I878" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J878" s="4">
+        <v>8</v>
+      </c>
+      <c r="K878" s="8">
+        <f>IFERROR(VLOOKUP(I878, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L878" s="9">
+        <f t="shared" si="14"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="879" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A879" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F879" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G879, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA 2000</v>
+      </c>
+      <c r="G879" s="1">
+        <v>4155</v>
+      </c>
+      <c r="H879" s="2">
+        <v>822</v>
+      </c>
+      <c r="I879" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J879" s="4">
+        <v>8</v>
+      </c>
+      <c r="K879" s="8">
+        <f>IFERROR(VLOOKUP(I879, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L879" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="880" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A880" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F880" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G880, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA 2000</v>
+      </c>
+      <c r="G880" s="1">
+        <v>4155</v>
+      </c>
+      <c r="H880" s="2">
+        <v>822</v>
+      </c>
+      <c r="I880" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J880" s="4">
+        <v>10</v>
+      </c>
+      <c r="K880" s="8">
+        <f>IFERROR(VLOOKUP(I880, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L880" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="881" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A881" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F881" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G881, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA 2000</v>
+      </c>
+      <c r="G881" s="1">
+        <v>4155</v>
+      </c>
+      <c r="H881" s="2">
+        <v>822</v>
+      </c>
+      <c r="I881" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J881" s="4">
+        <v>16</v>
+      </c>
+      <c r="K881" s="8">
+        <f>IFERROR(VLOOKUP(I881, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L881" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="882" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A882" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F882" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G882, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ROSARITO</v>
+      </c>
+      <c r="G882" s="1">
+        <v>4187</v>
+      </c>
+      <c r="H882" s="2">
+        <v>823</v>
+      </c>
+      <c r="I882" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J882" s="4">
+        <v>8</v>
+      </c>
+      <c r="K882" s="8">
+        <f>IFERROR(VLOOKUP(I882, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L882" s="9">
+        <f t="shared" si="14"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="883" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A883" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F883" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G883, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ROSARITO</v>
+      </c>
+      <c r="G883" s="1">
+        <v>4187</v>
+      </c>
+      <c r="H883" s="2">
+        <v>823</v>
+      </c>
+      <c r="I883" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J883" s="4">
+        <v>10</v>
+      </c>
+      <c r="K883" s="8">
+        <f>IFERROR(VLOOKUP(I883, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L883" s="9">
+        <f t="shared" si="14"/>
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="884" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A884" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F884" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G884, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ROSARITO</v>
+      </c>
+      <c r="G884" s="1">
+        <v>4187</v>
+      </c>
+      <c r="H884" s="2">
+        <v>823</v>
+      </c>
+      <c r="I884" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J884" s="4">
+        <v>8</v>
+      </c>
+      <c r="K884" s="8">
+        <f>IFERROR(VLOOKUP(I884, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L884" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="885" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A885" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F885" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G885, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ROSARITO</v>
+      </c>
+      <c r="G885" s="1">
+        <v>4187</v>
+      </c>
+      <c r="H885" s="2">
+        <v>823</v>
+      </c>
+      <c r="I885" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J885" s="4">
+        <v>20</v>
+      </c>
+      <c r="K885" s="8">
+        <f>IFERROR(VLOOKUP(I885, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L885" s="9">
+        <f t="shared" si="14"/>
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="886" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A886" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F886" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G886, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ROSARITO</v>
+      </c>
+      <c r="G886" s="1">
+        <v>4187</v>
+      </c>
+      <c r="H886" s="2">
+        <v>823</v>
+      </c>
+      <c r="I886" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J886" s="4">
+        <v>16</v>
+      </c>
+      <c r="K886" s="8">
+        <f>IFERROR(VLOOKUP(I886, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L886" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="887" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A887" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F887" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G887, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TECATE GARITA</v>
+      </c>
+      <c r="G887" s="1">
+        <v>5295</v>
+      </c>
+      <c r="H887" s="2">
+        <v>824</v>
+      </c>
+      <c r="I887" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J887" s="4">
+        <v>8</v>
+      </c>
+      <c r="K887" s="8">
+        <f>IFERROR(VLOOKUP(I887, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L887" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="888" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A888" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F888" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G888, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TECATE GARITA</v>
+      </c>
+      <c r="G888" s="1">
+        <v>5295</v>
+      </c>
+      <c r="H888" s="2">
+        <v>824</v>
+      </c>
+      <c r="I888" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J888" s="4">
+        <v>10</v>
+      </c>
+      <c r="K888" s="8">
+        <f>IFERROR(VLOOKUP(I888, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L888" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="889" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A889" s="54">
+        <v>46205</v>
+      </c>
+      <c r="F889" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G889, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TECATE GARITA</v>
+      </c>
+      <c r="G889" s="1">
+        <v>5295</v>
+      </c>
+      <c r="H889" s="2">
+        <v>824</v>
+      </c>
+      <c r="I889" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J889" s="4">
+        <v>16</v>
+      </c>
+      <c r="K889" s="8">
+        <f>IFERROR(VLOOKUP(I889, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L889" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="890" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A890" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F890" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G890, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA 2000</v>
+      </c>
+      <c r="G890" s="1">
+        <v>4155</v>
+      </c>
+      <c r="H890" s="2">
+        <v>825</v>
+      </c>
+      <c r="I890" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J890" s="4">
+        <v>8</v>
+      </c>
+      <c r="K890" s="8">
+        <f>IFERROR(VLOOKUP(I890, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L890" s="9">
+        <f t="shared" si="14"/>
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="891" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A891" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F891" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G891, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G891" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H891" s="2">
+        <v>826</v>
+      </c>
+      <c r="I891" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J891" s="4">
+        <v>4</v>
+      </c>
+      <c r="K891" s="8">
+        <f>IFERROR(VLOOKUP(I891, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L891" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="892" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A892" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F892" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G892, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC TIJUANA HIPODROMO</v>
+      </c>
+      <c r="G892" s="1">
+        <v>4011</v>
+      </c>
+      <c r="H892" s="2">
+        <v>826</v>
+      </c>
+      <c r="I892" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J892" s="4">
+        <v>6</v>
+      </c>
+      <c r="K892" s="8">
+        <f>IFERROR(VLOOKUP(I892, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L892" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="893" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A893" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F893" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G893, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G893" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H893" s="2">
+        <v>827</v>
+      </c>
+      <c r="I893" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J893" s="4">
+        <v>4</v>
+      </c>
+      <c r="K893" s="8">
+        <f>IFERROR(VLOOKUP(I893, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L893" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="894" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A894" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F894" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G894, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC DIAZ ORDAZ</v>
+      </c>
+      <c r="G894" s="1">
+        <v>3664</v>
+      </c>
+      <c r="H894" s="2">
+        <v>827</v>
+      </c>
+      <c r="I894" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J894" s="4">
+        <v>6</v>
+      </c>
+      <c r="K894" s="8">
+        <f>IFERROR(VLOOKUP(I894, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L894" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="895" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A895" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F895" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G895, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G895" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H895" s="2">
+        <v>828</v>
+      </c>
+      <c r="I895" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J895" s="4">
+        <v>4</v>
+      </c>
+      <c r="K895" s="8">
+        <f>IFERROR(VLOOKUP(I895, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L895" s="9">
+        <f t="shared" si="14"/>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="896" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A896" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F896" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G896, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC MACROPLAZA INSURGENTES</v>
+      </c>
+      <c r="G896" s="1">
+        <v>2023</v>
+      </c>
+      <c r="H896" s="2">
+        <v>828</v>
+      </c>
+      <c r="I896" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J896" s="4">
+        <v>6</v>
+      </c>
+      <c r="K896" s="8">
+        <f>IFERROR(VLOOKUP(I896, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L896" s="9">
+        <f t="shared" si="14"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="897" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A897" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F897" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G897, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA</v>
+      </c>
+      <c r="G897" s="1">
+        <v>3015</v>
+      </c>
+      <c r="H897" s="2">
+        <v>829</v>
+      </c>
+      <c r="I897" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J897" s="4">
+        <v>10</v>
+      </c>
+      <c r="K897" s="8">
+        <f>IFERROR(VLOOKUP(I897, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L897" s="9">
+        <f t="shared" si="14"/>
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="898" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A898" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F898" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G898, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA</v>
+      </c>
+      <c r="G898" s="1">
+        <v>3015</v>
+      </c>
+      <c r="H898" s="2">
+        <v>829</v>
+      </c>
+      <c r="I898" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J898" s="4">
+        <v>8</v>
+      </c>
+      <c r="K898" s="8">
+        <f>IFERROR(VLOOKUP(I898, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L898" s="9">
+        <f t="shared" si="14"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="899" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A899" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F899" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G899, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA</v>
+      </c>
+      <c r="G899" s="1">
+        <v>3015</v>
+      </c>
+      <c r="H899" s="2">
+        <v>829</v>
+      </c>
+      <c r="I899" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J899" s="4">
+        <v>10</v>
+      </c>
+      <c r="K899" s="8">
+        <f>IFERROR(VLOOKUP(I899, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L899" s="9">
+        <f t="shared" si="14"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="900" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A900" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F900" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G900, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA</v>
+      </c>
+      <c r="G900" s="1">
+        <v>3015</v>
+      </c>
+      <c r="H900" s="2">
+        <v>829</v>
+      </c>
+      <c r="I900" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J900" s="4">
+        <v>16</v>
+      </c>
+      <c r="K900" s="8">
+        <f>IFERROR(VLOOKUP(I900, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L900" s="9">
+        <f t="shared" si="14"/>
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="901" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A901" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F901" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G901, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA CENTRO</v>
+      </c>
+      <c r="G901" s="1">
+        <v>2947</v>
+      </c>
+      <c r="H901" s="2">
+        <v>830</v>
+      </c>
+      <c r="I901" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J901" s="4">
+        <v>4</v>
+      </c>
+      <c r="K901" s="8">
+        <f>IFERROR(VLOOKUP(I901, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>167</v>
+      </c>
+      <c r="L901" s="9">
+        <f t="shared" ref="L901:L905" si="15">K901*J901</f>
+        <v>668</v>
+      </c>
+    </row>
+    <row r="902" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A902" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F902" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G902, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA CENTRO</v>
+      </c>
+      <c r="G902" s="1">
+        <v>2947</v>
+      </c>
+      <c r="H902" s="2">
+        <v>830</v>
+      </c>
+      <c r="I902" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J902" s="4">
+        <v>6</v>
+      </c>
+      <c r="K902" s="8">
+        <f>IFERROR(VLOOKUP(I902, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>113</v>
+      </c>
+      <c r="L902" s="9">
+        <f t="shared" si="15"/>
+        <v>678</v>
+      </c>
+    </row>
+    <row r="903" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A903" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F903" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G903, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA CENTRO</v>
+      </c>
+      <c r="G903" s="1">
+        <v>2947</v>
+      </c>
+      <c r="H903" s="2">
+        <v>830</v>
+      </c>
+      <c r="I903" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J903" s="4">
+        <v>8</v>
+      </c>
+      <c r="K903" s="8">
+        <f>IFERROR(VLOOKUP(I903, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>151</v>
+      </c>
+      <c r="L903" s="9">
+        <f t="shared" si="15"/>
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="904" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A904" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F904" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G904, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA CENTRO</v>
+      </c>
+      <c r="G904" s="1">
+        <v>2947</v>
+      </c>
+      <c r="H904" s="2">
+        <v>830</v>
+      </c>
+      <c r="I904" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J904" s="4">
+        <v>10</v>
+      </c>
+      <c r="K904" s="8">
+        <f>IFERROR(VLOOKUP(I904, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>95</v>
+      </c>
+      <c r="L904" s="9">
+        <f t="shared" si="15"/>
+        <v>950</v>
+      </c>
+    </row>
+    <row r="905" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A905" s="54">
+        <v>46206</v>
+      </c>
+      <c r="F905" s="7" t="str">
+        <f>IFERROR(VLOOKUP(G905, data!A:B, 2, FALSE), "Tienda")</f>
+        <v>SC ENSENADA CENTRO</v>
+      </c>
+      <c r="G905" s="1">
+        <v>2947</v>
+      </c>
+      <c r="H905" s="2">
+        <v>830</v>
+      </c>
+      <c r="I905" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J905" s="4">
+        <v>16</v>
+      </c>
+      <c r="K905" s="8">
+        <f>IFERROR(VLOOKUP(I905, data!E:F, 2, FALSE), "Precio Unidad")</f>
+        <v>63</v>
+      </c>
+      <c r="L905" s="9">
+        <f t="shared" si="15"/>
+        <v>1008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>